<commit_message>
Added script and changed some columns in excel
</commit_message>
<xml_diff>
--- a/almarazflores_Ex3A_tables.xlsx
+++ b/almarazflores_Ex3A_tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julissaalmarazflores\Documents\DATA_labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FEF8BC-8A8E-42D0-B2F7-E7CB4A44CAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC70A462-A178-455D-8195-8FB57A508113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>ClientID</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t>Address</t>
   </si>
   <si>
@@ -82,10 +79,10 @@
     <t>Amount</t>
   </si>
   <si>
-    <t>Method</t>
-  </si>
-  <si>
     <t>WalkDogID</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
   </si>
 </sst>
 </file>
@@ -433,16 +430,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.08984375" customWidth="1"/>
     <col min="3" max="3" width="9.54296875" customWidth="1"/>
     <col min="4" max="4" width="9.90625" customWidth="1"/>
-    <col min="5" max="5" width="9.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -457,9 +453,6 @@
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -474,16 +467,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>0</v>
@@ -501,19 +494,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -531,22 +524,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -564,13 +557,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>